<commit_message>
Cortrecion en Cenco, copi, y cambios varios
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_copi.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_copi.xlsx
@@ -526,12 +526,12 @@
     <col width="2" customWidth="1" min="1" max="1"/>
     <col width="2" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="17" customWidth="1" min="8" max="8"/>
-    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1"/>
@@ -643,7 +643,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>11/11/2025</t>
+          <t>19/11/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2518,27 +2518,35 @@
     <row r="101">
       <c r="C101" s="10" t="inlineStr">
         <is>
-          <t>Nota de reintegro</t>
+          <t>Devolucion</t>
         </is>
       </c>
       <c r="D101" s="10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>5009220606</t>
         </is>
       </c>
       <c r="E101" s="6" t="n">
-        <v>359576835</v>
-      </c>
-      <c r="F101" s="10" t="inlineStr"/>
+        <v>-21203</v>
+      </c>
+      <c r="F101" s="10" t="inlineStr">
+        <is>
+          <t>AVERIA</t>
+        </is>
+      </c>
       <c r="G101" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>522</t>
         </is>
       </c>
       <c r="H101" s="6" t="n">
-        <v>359576835</v>
-      </c>
-      <c r="I101" s="11" t="inlineStr"/>
+        <v>-21203</v>
+      </c>
+      <c r="I101" s="11" t="inlineStr">
+        <is>
+          <t>AVERIA 5009220606</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="C102" s="10" t="inlineStr">
@@ -2548,11 +2556,11 @@
       </c>
       <c r="D102" s="10" t="inlineStr">
         <is>
-          <t>5009220606</t>
+          <t>5009224095</t>
         </is>
       </c>
       <c r="E102" s="6" t="n">
-        <v>-21203</v>
+        <v>-441984</v>
       </c>
       <c r="F102" s="10" t="inlineStr">
         <is>
@@ -2565,11 +2573,11 @@
         </is>
       </c>
       <c r="H102" s="6" t="n">
-        <v>-21203</v>
+        <v>-441984</v>
       </c>
       <c r="I102" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009220606</t>
+          <t>AVERIA 5009224095</t>
         </is>
       </c>
     </row>
@@ -2581,11 +2589,11 @@
       </c>
       <c r="D103" s="10" t="inlineStr">
         <is>
-          <t>5009224095</t>
+          <t>5009224444</t>
         </is>
       </c>
       <c r="E103" s="6" t="n">
-        <v>-441984</v>
+        <v>-292047</v>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
@@ -2598,11 +2606,11 @@
         </is>
       </c>
       <c r="H103" s="6" t="n">
-        <v>-441984</v>
+        <v>-292047</v>
       </c>
       <c r="I103" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009224095</t>
+          <t>AVERIA 5009224444</t>
         </is>
       </c>
     </row>
@@ -2614,11 +2622,11 @@
       </c>
       <c r="D104" s="10" t="inlineStr">
         <is>
-          <t>5009224444</t>
+          <t>5009224690</t>
         </is>
       </c>
       <c r="E104" s="6" t="n">
-        <v>-292047</v>
+        <v>-18852</v>
       </c>
       <c r="F104" s="10" t="inlineStr">
         <is>
@@ -2631,11 +2639,11 @@
         </is>
       </c>
       <c r="H104" s="6" t="n">
-        <v>-292047</v>
+        <v>-18852</v>
       </c>
       <c r="I104" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009224444</t>
+          <t>AVERIA 5009224690</t>
         </is>
       </c>
     </row>
@@ -2647,11 +2655,11 @@
       </c>
       <c r="D105" s="10" t="inlineStr">
         <is>
-          <t>5009224690</t>
+          <t>5009224702</t>
         </is>
       </c>
       <c r="E105" s="6" t="n">
-        <v>-18852</v>
+        <v>-15200</v>
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
@@ -2664,11 +2672,11 @@
         </is>
       </c>
       <c r="H105" s="6" t="n">
-        <v>-18852</v>
+        <v>-15200</v>
       </c>
       <c r="I105" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009224690</t>
+          <t>AVERIA 5009224702</t>
         </is>
       </c>
     </row>
@@ -2680,11 +2688,11 @@
       </c>
       <c r="D106" s="10" t="inlineStr">
         <is>
-          <t>5009224702</t>
+          <t>5009224750</t>
         </is>
       </c>
       <c r="E106" s="6" t="n">
-        <v>-15200</v>
+        <v>-2217111</v>
       </c>
       <c r="F106" s="10" t="inlineStr">
         <is>
@@ -2697,11 +2705,11 @@
         </is>
       </c>
       <c r="H106" s="6" t="n">
-        <v>-15200</v>
+        <v>-2217111</v>
       </c>
       <c r="I106" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009224702</t>
+          <t>AVERIA 5009224750</t>
         </is>
       </c>
     </row>
@@ -2713,11 +2721,11 @@
       </c>
       <c r="D107" s="10" t="inlineStr">
         <is>
-          <t>5009224750</t>
+          <t>5009225047</t>
         </is>
       </c>
       <c r="E107" s="6" t="n">
-        <v>-2217111</v>
+        <v>-8175</v>
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
@@ -2730,11 +2738,11 @@
         </is>
       </c>
       <c r="H107" s="6" t="n">
-        <v>-2217111</v>
+        <v>-8175</v>
       </c>
       <c r="I107" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009224750</t>
+          <t>AVERIA 5009225047</t>
         </is>
       </c>
     </row>
@@ -2746,11 +2754,11 @@
       </c>
       <c r="D108" s="10" t="inlineStr">
         <is>
-          <t>5009225047</t>
+          <t>5009225048</t>
         </is>
       </c>
       <c r="E108" s="6" t="n">
-        <v>-8175</v>
+        <v>-1083655</v>
       </c>
       <c r="F108" s="10" t="inlineStr">
         <is>
@@ -2763,11 +2771,11 @@
         </is>
       </c>
       <c r="H108" s="6" t="n">
-        <v>-8175</v>
+        <v>-1083655</v>
       </c>
       <c r="I108" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009225047</t>
+          <t>AVERIA 5009225048</t>
         </is>
       </c>
     </row>
@@ -2779,11 +2787,11 @@
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t>5009225048</t>
+          <t>5009225109</t>
         </is>
       </c>
       <c r="E109" s="6" t="n">
-        <v>-1083655</v>
+        <v>-86077</v>
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
@@ -2796,11 +2804,11 @@
         </is>
       </c>
       <c r="H109" s="6" t="n">
-        <v>-1083655</v>
+        <v>-86077</v>
       </c>
       <c r="I109" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009225048</t>
+          <t>AVERIA 5009225109</t>
         </is>
       </c>
     </row>
@@ -2812,11 +2820,11 @@
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t>5009225109</t>
+          <t>5009225176</t>
         </is>
       </c>
       <c r="E110" s="6" t="n">
-        <v>-86077</v>
+        <v>-106960</v>
       </c>
       <c r="F110" s="10" t="inlineStr">
         <is>
@@ -2829,11 +2837,11 @@
         </is>
       </c>
       <c r="H110" s="6" t="n">
-        <v>-86077</v>
+        <v>-106960</v>
       </c>
       <c r="I110" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009225109</t>
+          <t>AVERIA 5009225176</t>
         </is>
       </c>
     </row>
@@ -2845,11 +2853,11 @@
       </c>
       <c r="D111" s="10" t="inlineStr">
         <is>
-          <t>5009225176</t>
+          <t>5009225178</t>
         </is>
       </c>
       <c r="E111" s="6" t="n">
-        <v>-106960</v>
+        <v>-83875</v>
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
@@ -2862,11 +2870,11 @@
         </is>
       </c>
       <c r="H111" s="6" t="n">
-        <v>-106960</v>
+        <v>-83875</v>
       </c>
       <c r="I111" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009225176</t>
+          <t>AVERIA 5009225178</t>
         </is>
       </c>
     </row>
@@ -2878,11 +2886,11 @@
       </c>
       <c r="D112" s="10" t="inlineStr">
         <is>
-          <t>5009225178</t>
+          <t>5009225251</t>
         </is>
       </c>
       <c r="E112" s="6" t="n">
-        <v>-83875</v>
+        <v>-195679</v>
       </c>
       <c r="F112" s="10" t="inlineStr">
         <is>
@@ -2895,11 +2903,11 @@
         </is>
       </c>
       <c r="H112" s="6" t="n">
-        <v>-83875</v>
+        <v>-195679</v>
       </c>
       <c r="I112" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009225178</t>
+          <t>AVERIA 5009225251</t>
         </is>
       </c>
     </row>
@@ -2911,11 +2919,11 @@
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t>5009225251</t>
+          <t>5009225361</t>
         </is>
       </c>
       <c r="E113" s="6" t="n">
-        <v>-195679</v>
+        <v>-206032</v>
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
@@ -2928,11 +2936,11 @@
         </is>
       </c>
       <c r="H113" s="6" t="n">
-        <v>-195679</v>
+        <v>-206032</v>
       </c>
       <c r="I113" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009225251</t>
+          <t>AVERIA 5009225361</t>
         </is>
       </c>
     </row>
@@ -2944,11 +2952,11 @@
       </c>
       <c r="D114" s="10" t="inlineStr">
         <is>
-          <t>5009225361</t>
+          <t>5009231150</t>
         </is>
       </c>
       <c r="E114" s="6" t="n">
-        <v>-206032</v>
+        <v>-3115</v>
       </c>
       <c r="F114" s="10" t="inlineStr">
         <is>
@@ -2961,11 +2969,11 @@
         </is>
       </c>
       <c r="H114" s="6" t="n">
-        <v>-206032</v>
+        <v>-3115</v>
       </c>
       <c r="I114" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009225361</t>
+          <t>AVERIA 5009231150</t>
         </is>
       </c>
     </row>
@@ -2977,11 +2985,11 @@
       </c>
       <c r="D115" s="10" t="inlineStr">
         <is>
-          <t>5009231150</t>
+          <t>5009231161</t>
         </is>
       </c>
       <c r="E115" s="6" t="n">
-        <v>-3115</v>
+        <v>-18852</v>
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
@@ -2994,11 +3002,11 @@
         </is>
       </c>
       <c r="H115" s="6" t="n">
-        <v>-3115</v>
+        <v>-18852</v>
       </c>
       <c r="I115" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009231150</t>
+          <t>AVERIA 5009231161</t>
         </is>
       </c>
     </row>
@@ -3010,11 +3018,11 @@
       </c>
       <c r="D116" s="10" t="inlineStr">
         <is>
-          <t>5009231161</t>
+          <t>5009231162</t>
         </is>
       </c>
       <c r="E116" s="6" t="n">
-        <v>-18852</v>
+        <v>-2743</v>
       </c>
       <c r="F116" s="10" t="inlineStr">
         <is>
@@ -3027,11 +3035,11 @@
         </is>
       </c>
       <c r="H116" s="6" t="n">
-        <v>-18852</v>
+        <v>-2743</v>
       </c>
       <c r="I116" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009231161</t>
+          <t>AVERIA 5009231162</t>
         </is>
       </c>
     </row>
@@ -3043,11 +3051,11 @@
       </c>
       <c r="D117" s="10" t="inlineStr">
         <is>
-          <t>5009231162</t>
+          <t>5009231192</t>
         </is>
       </c>
       <c r="E117" s="6" t="n">
-        <v>-2743</v>
+        <v>-131965</v>
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
@@ -3060,11 +3068,11 @@
         </is>
       </c>
       <c r="H117" s="6" t="n">
-        <v>-2743</v>
+        <v>-131965</v>
       </c>
       <c r="I117" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009231162</t>
+          <t>AVERIA 5009231192</t>
         </is>
       </c>
     </row>
@@ -3076,11 +3084,11 @@
       </c>
       <c r="D118" s="10" t="inlineStr">
         <is>
-          <t>5009231192</t>
+          <t>5009231193</t>
         </is>
       </c>
       <c r="E118" s="6" t="n">
-        <v>-131965</v>
+        <v>-28261</v>
       </c>
       <c r="F118" s="10" t="inlineStr">
         <is>
@@ -3093,11 +3101,11 @@
         </is>
       </c>
       <c r="H118" s="6" t="n">
-        <v>-131965</v>
+        <v>-28261</v>
       </c>
       <c r="I118" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009231192</t>
+          <t>AVERIA 5009231193</t>
         </is>
       </c>
     </row>
@@ -3109,11 +3117,11 @@
       </c>
       <c r="D119" s="10" t="inlineStr">
         <is>
-          <t>5009231193</t>
+          <t>5009231195</t>
         </is>
       </c>
       <c r="E119" s="6" t="n">
-        <v>-28261</v>
+        <v>-576910</v>
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
@@ -3126,11 +3134,11 @@
         </is>
       </c>
       <c r="H119" s="6" t="n">
-        <v>-28261</v>
+        <v>-576910</v>
       </c>
       <c r="I119" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009231193</t>
+          <t>AVERIA 5009231195</t>
         </is>
       </c>
     </row>
@@ -3142,11 +3150,11 @@
       </c>
       <c r="D120" s="10" t="inlineStr">
         <is>
-          <t>5009231195</t>
+          <t>5009231196</t>
         </is>
       </c>
       <c r="E120" s="6" t="n">
-        <v>-576910</v>
+        <v>-1670389</v>
       </c>
       <c r="F120" s="10" t="inlineStr">
         <is>
@@ -3159,11 +3167,11 @@
         </is>
       </c>
       <c r="H120" s="6" t="n">
-        <v>-576910</v>
+        <v>-1670389</v>
       </c>
       <c r="I120" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009231195</t>
+          <t>AVERIA 5009231196</t>
         </is>
       </c>
     </row>
@@ -3175,11 +3183,11 @@
       </c>
       <c r="D121" s="10" t="inlineStr">
         <is>
-          <t>5009231196</t>
+          <t>5009237069</t>
         </is>
       </c>
       <c r="E121" s="6" t="n">
-        <v>-1670389</v>
+        <v>-15200</v>
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
@@ -3192,44 +3200,44 @@
         </is>
       </c>
       <c r="H121" s="6" t="n">
-        <v>-1670389</v>
+        <v>-15200</v>
       </c>
       <c r="I121" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009231196</t>
+          <t>AVERIA 5009237069</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="C122" s="10" t="inlineStr">
         <is>
-          <t>Devolucion</t>
+          <t>Nota</t>
         </is>
       </c>
       <c r="D122" s="10" t="inlineStr">
         <is>
-          <t>5009237069</t>
+          <t>NOTA DEVOLUCIÓN</t>
         </is>
       </c>
       <c r="E122" s="6" t="n">
-        <v>-15200</v>
+        <v>-145827858</v>
       </c>
       <c r="F122" s="10" t="inlineStr">
         <is>
-          <t>AVERIA</t>
+          <t>DESCUENTO</t>
         </is>
       </c>
       <c r="G122" s="10" t="inlineStr">
         <is>
-          <t>522</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H122" s="6" t="n">
-        <v>-15200</v>
+        <v>-145827858</v>
       </c>
       <c r="I122" s="11" t="inlineStr">
         <is>
-          <t>AVERIA 5009237069</t>
+          <t>DESCUENTO NOTA DEVOLUCIÓN</t>
         </is>
       </c>
     </row>
@@ -3245,7 +3253,7 @@
         </is>
       </c>
       <c r="E123" s="6" t="n">
-        <v>-145827858</v>
+        <v>-58271729</v>
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
@@ -3258,7 +3266,7 @@
         </is>
       </c>
       <c r="H123" s="6" t="n">
-        <v>-145827858</v>
+        <v>-58271729</v>
       </c>
       <c r="I123" s="11" t="inlineStr">
         <is>
@@ -3274,11 +3282,11 @@
       </c>
       <c r="D124" s="10" t="inlineStr">
         <is>
-          <t>NOTA DEVOLUCIÓN</t>
+          <t>Nota</t>
         </is>
       </c>
       <c r="E124" s="6" t="n">
-        <v>-58271729</v>
+        <v>-648119521</v>
       </c>
       <c r="F124" s="10" t="inlineStr">
         <is>
@@ -3291,27 +3299,27 @@
         </is>
       </c>
       <c r="H124" s="6" t="n">
-        <v>-58271729</v>
+        <v>-648119521</v>
       </c>
       <c r="I124" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO NOTA DEVOLUCIÓN</t>
+          <t>Cumpl.acuerdo información mes 08 2025 -Unilever</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="C125" s="10" t="inlineStr">
         <is>
-          <t>Nota</t>
+          <t>Reduc Factura Compra</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>PMP1282241</t>
         </is>
       </c>
       <c r="E125" s="6" t="n">
-        <v>-648119521</v>
+        <v>-293425</v>
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
@@ -3324,11 +3332,11 @@
         </is>
       </c>
       <c r="H125" s="6" t="n">
-        <v>-648119521</v>
+        <v>-293425</v>
       </c>
       <c r="I125" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO nan</t>
+          <t>DESCUENTO PMP1282241</t>
         </is>
       </c>
     </row>
@@ -3340,11 +3348,11 @@
       </c>
       <c r="D126" s="10" t="inlineStr">
         <is>
-          <t>PMP1282241</t>
+          <t>PMP1282247</t>
         </is>
       </c>
       <c r="E126" s="6" t="n">
-        <v>-293425</v>
+        <v>-1413822</v>
       </c>
       <c r="F126" s="10" t="inlineStr">
         <is>
@@ -3357,11 +3365,11 @@
         </is>
       </c>
       <c r="H126" s="6" t="n">
-        <v>-293425</v>
+        <v>-1413822</v>
       </c>
       <c r="I126" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1282241</t>
+          <t>DESCUENTO PMP1282247</t>
         </is>
       </c>
     </row>
@@ -3373,11 +3381,11 @@
       </c>
       <c r="D127" s="10" t="inlineStr">
         <is>
-          <t>PMP1282247</t>
+          <t>PMP1284756</t>
         </is>
       </c>
       <c r="E127" s="6" t="n">
-        <v>-1413822</v>
+        <v>-168578</v>
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
@@ -3390,11 +3398,11 @@
         </is>
       </c>
       <c r="H127" s="6" t="n">
-        <v>-1413822</v>
+        <v>-168578</v>
       </c>
       <c r="I127" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1282247</t>
+          <t>DESCUENTO PMP1284756</t>
         </is>
       </c>
     </row>
@@ -3406,11 +3414,11 @@
       </c>
       <c r="D128" s="10" t="inlineStr">
         <is>
-          <t>PMP1284756</t>
+          <t>PMP1285097</t>
         </is>
       </c>
       <c r="E128" s="6" t="n">
-        <v>-168578</v>
+        <v>-669705</v>
       </c>
       <c r="F128" s="10" t="inlineStr">
         <is>
@@ -3423,11 +3431,11 @@
         </is>
       </c>
       <c r="H128" s="6" t="n">
-        <v>-168578</v>
+        <v>-669705</v>
       </c>
       <c r="I128" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1284756</t>
+          <t>DESCUENTO PMP1285097</t>
         </is>
       </c>
     </row>
@@ -3439,11 +3447,11 @@
       </c>
       <c r="D129" s="10" t="inlineStr">
         <is>
-          <t>PMP1285097</t>
+          <t>PMP1285525</t>
         </is>
       </c>
       <c r="E129" s="6" t="n">
-        <v>-669705</v>
+        <v>-8631817</v>
       </c>
       <c r="F129" s="10" t="inlineStr">
         <is>
@@ -3456,11 +3464,11 @@
         </is>
       </c>
       <c r="H129" s="6" t="n">
-        <v>-669705</v>
+        <v>-8631817</v>
       </c>
       <c r="I129" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1285097</t>
+          <t>DESCUENTO PMP1285525</t>
         </is>
       </c>
     </row>
@@ -3472,11 +3480,11 @@
       </c>
       <c r="D130" s="10" t="inlineStr">
         <is>
-          <t>PMP1285525</t>
+          <t>PMP1287684</t>
         </is>
       </c>
       <c r="E130" s="6" t="n">
-        <v>-8631817</v>
+        <v>-29736</v>
       </c>
       <c r="F130" s="10" t="inlineStr">
         <is>
@@ -3489,11 +3497,11 @@
         </is>
       </c>
       <c r="H130" s="6" t="n">
-        <v>-8631817</v>
+        <v>-29736</v>
       </c>
       <c r="I130" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1285525</t>
+          <t>DESCUENTO PMP1287684</t>
         </is>
       </c>
     </row>
@@ -3505,11 +3513,11 @@
       </c>
       <c r="D131" s="10" t="inlineStr">
         <is>
-          <t>PMP1287684</t>
+          <t>PMP1287685</t>
         </is>
       </c>
       <c r="E131" s="6" t="n">
-        <v>-29736</v>
+        <v>-2323867</v>
       </c>
       <c r="F131" s="10" t="inlineStr">
         <is>
@@ -3522,11 +3530,11 @@
         </is>
       </c>
       <c r="H131" s="6" t="n">
-        <v>-29736</v>
+        <v>-2323867</v>
       </c>
       <c r="I131" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1287684</t>
+          <t>DESCUENTO PMP1287685</t>
         </is>
       </c>
     </row>
@@ -3538,11 +3546,11 @@
       </c>
       <c r="D132" s="10" t="inlineStr">
         <is>
-          <t>PMP1287685</t>
+          <t>PMP1287687</t>
         </is>
       </c>
       <c r="E132" s="6" t="n">
-        <v>-2323867</v>
+        <v>-1707987</v>
       </c>
       <c r="F132" s="10" t="inlineStr">
         <is>
@@ -3555,11 +3563,11 @@
         </is>
       </c>
       <c r="H132" s="6" t="n">
-        <v>-2323867</v>
+        <v>-1707987</v>
       </c>
       <c r="I132" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1287685</t>
+          <t>DESCUENTO PMP1287687</t>
         </is>
       </c>
     </row>
@@ -3571,11 +3579,11 @@
       </c>
       <c r="D133" s="10" t="inlineStr">
         <is>
-          <t>PMP1287687</t>
+          <t>PMP1287690</t>
         </is>
       </c>
       <c r="E133" s="6" t="n">
-        <v>-1707987</v>
+        <v>-306035</v>
       </c>
       <c r="F133" s="10" t="inlineStr">
         <is>
@@ -3588,11 +3596,11 @@
         </is>
       </c>
       <c r="H133" s="6" t="n">
-        <v>-1707987</v>
+        <v>-306035</v>
       </c>
       <c r="I133" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1287687</t>
+          <t>DESCUENTO PMP1287690</t>
         </is>
       </c>
     </row>
@@ -3604,11 +3612,11 @@
       </c>
       <c r="D134" s="10" t="inlineStr">
         <is>
-          <t>PMP1287690</t>
+          <t>PMP1287691</t>
         </is>
       </c>
       <c r="E134" s="6" t="n">
-        <v>-306035</v>
+        <v>-88972</v>
       </c>
       <c r="F134" s="10" t="inlineStr">
         <is>
@@ -3621,11 +3629,11 @@
         </is>
       </c>
       <c r="H134" s="6" t="n">
-        <v>-306035</v>
+        <v>-88972</v>
       </c>
       <c r="I134" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1287690</t>
+          <t>DESCUENTO PMP1287691</t>
         </is>
       </c>
     </row>
@@ -3637,11 +3645,11 @@
       </c>
       <c r="D135" s="10" t="inlineStr">
         <is>
-          <t>PMP1287691</t>
+          <t>PMP1287693</t>
         </is>
       </c>
       <c r="E135" s="6" t="n">
-        <v>-88972</v>
+        <v>-588272</v>
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
@@ -3654,11 +3662,11 @@
         </is>
       </c>
       <c r="H135" s="6" t="n">
-        <v>-88972</v>
+        <v>-588272</v>
       </c>
       <c r="I135" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1287691</t>
+          <t>DESCUENTO PMP1287693</t>
         </is>
       </c>
     </row>
@@ -3670,11 +3678,11 @@
       </c>
       <c r="D136" s="10" t="inlineStr">
         <is>
-          <t>PMP1287693</t>
+          <t>PMP1287697</t>
         </is>
       </c>
       <c r="E136" s="6" t="n">
-        <v>-588272</v>
+        <v>-280688</v>
       </c>
       <c r="F136" s="10" t="inlineStr">
         <is>
@@ -3687,11 +3695,11 @@
         </is>
       </c>
       <c r="H136" s="6" t="n">
-        <v>-588272</v>
+        <v>-280688</v>
       </c>
       <c r="I136" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1287693</t>
+          <t>DESCUENTO PMP1287697</t>
         </is>
       </c>
     </row>
@@ -3703,11 +3711,11 @@
       </c>
       <c r="D137" s="10" t="inlineStr">
         <is>
-          <t>PMP1287697</t>
+          <t>PMP1287698</t>
         </is>
       </c>
       <c r="E137" s="6" t="n">
-        <v>-280688</v>
+        <v>-85801</v>
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
@@ -3720,11 +3728,11 @@
         </is>
       </c>
       <c r="H137" s="6" t="n">
-        <v>-280688</v>
+        <v>-85801</v>
       </c>
       <c r="I137" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1287697</t>
+          <t>DESCUENTO PMP1287698</t>
         </is>
       </c>
     </row>
@@ -3736,11 +3744,11 @@
       </c>
       <c r="D138" s="10" t="inlineStr">
         <is>
-          <t>PMP1287698</t>
+          <t>PMP1288308</t>
         </is>
       </c>
       <c r="E138" s="6" t="n">
-        <v>-85801</v>
+        <v>-19823</v>
       </c>
       <c r="F138" s="10" t="inlineStr">
         <is>
@@ -3753,11 +3761,11 @@
         </is>
       </c>
       <c r="H138" s="6" t="n">
-        <v>-85801</v>
+        <v>-19823</v>
       </c>
       <c r="I138" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1287698</t>
+          <t>DESCUENTO PMP1288308</t>
         </is>
       </c>
     </row>
@@ -3769,11 +3777,11 @@
       </c>
       <c r="D139" s="10" t="inlineStr">
         <is>
-          <t>PMP1288308</t>
+          <t>PMP1288311</t>
         </is>
       </c>
       <c r="E139" s="6" t="n">
-        <v>-19823</v>
+        <v>-1974873</v>
       </c>
       <c r="F139" s="10" t="inlineStr">
         <is>
@@ -3786,11 +3794,11 @@
         </is>
       </c>
       <c r="H139" s="6" t="n">
-        <v>-19823</v>
+        <v>-1974873</v>
       </c>
       <c r="I139" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288308</t>
+          <t>DESCUENTO PMP1288311</t>
         </is>
       </c>
     </row>
@@ -3802,11 +3810,11 @@
       </c>
       <c r="D140" s="10" t="inlineStr">
         <is>
-          <t>PMP1288311</t>
+          <t>PMP1288312</t>
         </is>
       </c>
       <c r="E140" s="6" t="n">
-        <v>-1974873</v>
+        <v>-2615840</v>
       </c>
       <c r="F140" s="10" t="inlineStr">
         <is>
@@ -3819,11 +3827,11 @@
         </is>
       </c>
       <c r="H140" s="6" t="n">
-        <v>-1974873</v>
+        <v>-2615840</v>
       </c>
       <c r="I140" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288311</t>
+          <t>DESCUENTO PMP1288312</t>
         </is>
       </c>
     </row>
@@ -3835,11 +3843,11 @@
       </c>
       <c r="D141" s="10" t="inlineStr">
         <is>
-          <t>PMP1288312</t>
+          <t>PMP1288313</t>
         </is>
       </c>
       <c r="E141" s="6" t="n">
-        <v>-2615840</v>
+        <v>-494251</v>
       </c>
       <c r="F141" s="10" t="inlineStr">
         <is>
@@ -3852,11 +3860,11 @@
         </is>
       </c>
       <c r="H141" s="6" t="n">
-        <v>-2615840</v>
+        <v>-494251</v>
       </c>
       <c r="I141" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288312</t>
+          <t>DESCUENTO PMP1288313</t>
         </is>
       </c>
     </row>
@@ -3868,11 +3876,11 @@
       </c>
       <c r="D142" s="10" t="inlineStr">
         <is>
-          <t>PMP1288313</t>
+          <t>PMP1288316</t>
         </is>
       </c>
       <c r="E142" s="6" t="n">
-        <v>-494251</v>
+        <v>-463129</v>
       </c>
       <c r="F142" s="10" t="inlineStr">
         <is>
@@ -3885,11 +3893,11 @@
         </is>
       </c>
       <c r="H142" s="6" t="n">
-        <v>-494251</v>
+        <v>-463129</v>
       </c>
       <c r="I142" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288313</t>
+          <t>DESCUENTO PMP1288316</t>
         </is>
       </c>
     </row>
@@ -3901,11 +3909,11 @@
       </c>
       <c r="D143" s="10" t="inlineStr">
         <is>
-          <t>PMP1288316</t>
+          <t>PMP1288317</t>
         </is>
       </c>
       <c r="E143" s="6" t="n">
-        <v>-463129</v>
+        <v>-221194</v>
       </c>
       <c r="F143" s="10" t="inlineStr">
         <is>
@@ -3918,11 +3926,11 @@
         </is>
       </c>
       <c r="H143" s="6" t="n">
-        <v>-463129</v>
+        <v>-221194</v>
       </c>
       <c r="I143" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288316</t>
+          <t>DESCUENTO PMP1288317</t>
         </is>
       </c>
     </row>
@@ -3934,11 +3942,11 @@
       </c>
       <c r="D144" s="10" t="inlineStr">
         <is>
-          <t>PMP1288317</t>
+          <t>PMP1288320</t>
         </is>
       </c>
       <c r="E144" s="6" t="n">
-        <v>-221194</v>
+        <v>-3253412</v>
       </c>
       <c r="F144" s="10" t="inlineStr">
         <is>
@@ -3951,11 +3959,11 @@
         </is>
       </c>
       <c r="H144" s="6" t="n">
-        <v>-221194</v>
+        <v>-3253412</v>
       </c>
       <c r="I144" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288317</t>
+          <t>DESCUENTO PMP1288320</t>
         </is>
       </c>
     </row>
@@ -3967,11 +3975,11 @@
       </c>
       <c r="D145" s="10" t="inlineStr">
         <is>
-          <t>PMP1288320</t>
+          <t>PMP1288322</t>
         </is>
       </c>
       <c r="E145" s="6" t="n">
-        <v>-3253412</v>
+        <v>-261582</v>
       </c>
       <c r="F145" s="10" t="inlineStr">
         <is>
@@ -3984,11 +3992,11 @@
         </is>
       </c>
       <c r="H145" s="6" t="n">
-        <v>-3253412</v>
+        <v>-261582</v>
       </c>
       <c r="I145" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288320</t>
+          <t>DESCUENTO PMP1288322</t>
         </is>
       </c>
     </row>
@@ -4000,11 +4008,11 @@
       </c>
       <c r="D146" s="10" t="inlineStr">
         <is>
-          <t>PMP1288322</t>
+          <t>PMP1288323</t>
         </is>
       </c>
       <c r="E146" s="6" t="n">
-        <v>-261582</v>
+        <v>-500713</v>
       </c>
       <c r="F146" s="10" t="inlineStr">
         <is>
@@ -4017,11 +4025,11 @@
         </is>
       </c>
       <c r="H146" s="6" t="n">
-        <v>-261582</v>
+        <v>-500713</v>
       </c>
       <c r="I146" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288322</t>
+          <t>DESCUENTO PMP1288323</t>
         </is>
       </c>
     </row>
@@ -4033,11 +4041,11 @@
       </c>
       <c r="D147" s="10" t="inlineStr">
         <is>
-          <t>PMP1288323</t>
+          <t>PMP1288324</t>
         </is>
       </c>
       <c r="E147" s="6" t="n">
-        <v>-500713</v>
+        <v>-377591</v>
       </c>
       <c r="F147" s="10" t="inlineStr">
         <is>
@@ -4050,11 +4058,11 @@
         </is>
       </c>
       <c r="H147" s="6" t="n">
-        <v>-500713</v>
+        <v>-377591</v>
       </c>
       <c r="I147" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288323</t>
+          <t>DESCUENTO PMP1288324</t>
         </is>
       </c>
     </row>
@@ -4066,11 +4074,11 @@
       </c>
       <c r="D148" s="10" t="inlineStr">
         <is>
-          <t>PMP1288324</t>
+          <t>PMP1288444</t>
         </is>
       </c>
       <c r="E148" s="6" t="n">
-        <v>-377591</v>
+        <v>-104074</v>
       </c>
       <c r="F148" s="10" t="inlineStr">
         <is>
@@ -4083,11 +4091,11 @@
         </is>
       </c>
       <c r="H148" s="6" t="n">
-        <v>-377591</v>
+        <v>-104074</v>
       </c>
       <c r="I148" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288324</t>
+          <t>DESCUENTO PMP1288444</t>
         </is>
       </c>
     </row>
@@ -4099,11 +4107,11 @@
       </c>
       <c r="D149" s="10" t="inlineStr">
         <is>
-          <t>PMP1288444</t>
+          <t>PMP1288450</t>
         </is>
       </c>
       <c r="E149" s="6" t="n">
-        <v>-104074</v>
+        <v>-1821689</v>
       </c>
       <c r="F149" s="10" t="inlineStr">
         <is>
@@ -4116,11 +4124,11 @@
         </is>
       </c>
       <c r="H149" s="6" t="n">
-        <v>-104074</v>
+        <v>-1821689</v>
       </c>
       <c r="I149" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288444</t>
+          <t>DESCUENTO PMP1288450</t>
         </is>
       </c>
     </row>
@@ -4132,11 +4140,11 @@
       </c>
       <c r="D150" s="10" t="inlineStr">
         <is>
-          <t>PMP1288450</t>
+          <t>PMP1288451</t>
         </is>
       </c>
       <c r="E150" s="6" t="n">
-        <v>-1821689</v>
+        <v>-3344689</v>
       </c>
       <c r="F150" s="10" t="inlineStr">
         <is>
@@ -4149,11 +4157,11 @@
         </is>
       </c>
       <c r="H150" s="6" t="n">
-        <v>-1821689</v>
+        <v>-3344689</v>
       </c>
       <c r="I150" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288450</t>
+          <t>DESCUENTO PMP1288451</t>
         </is>
       </c>
     </row>
@@ -4165,11 +4173,11 @@
       </c>
       <c r="D151" s="10" t="inlineStr">
         <is>
-          <t>PMP1288451</t>
+          <t>PMP1288452</t>
         </is>
       </c>
       <c r="E151" s="6" t="n">
-        <v>-3344689</v>
+        <v>-12557407</v>
       </c>
       <c r="F151" s="10" t="inlineStr">
         <is>
@@ -4182,11 +4190,11 @@
         </is>
       </c>
       <c r="H151" s="6" t="n">
-        <v>-3344689</v>
+        <v>-12557407</v>
       </c>
       <c r="I151" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288451</t>
+          <t>DESCUENTO PMP1288452</t>
         </is>
       </c>
     </row>
@@ -4198,11 +4206,11 @@
       </c>
       <c r="D152" s="10" t="inlineStr">
         <is>
-          <t>PMP1288452</t>
+          <t>PMP1288453</t>
         </is>
       </c>
       <c r="E152" s="6" t="n">
-        <v>-12557407</v>
+        <v>-1758852</v>
       </c>
       <c r="F152" s="10" t="inlineStr">
         <is>
@@ -4215,11 +4223,11 @@
         </is>
       </c>
       <c r="H152" s="6" t="n">
-        <v>-12557407</v>
+        <v>-1758852</v>
       </c>
       <c r="I152" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288452</t>
+          <t>DESCUENTO PMP1288453</t>
         </is>
       </c>
     </row>
@@ -4231,11 +4239,11 @@
       </c>
       <c r="D153" s="10" t="inlineStr">
         <is>
-          <t>PMP1288453</t>
+          <t>PMP1288454</t>
         </is>
       </c>
       <c r="E153" s="6" t="n">
-        <v>-1758852</v>
+        <v>-4388718</v>
       </c>
       <c r="F153" s="10" t="inlineStr">
         <is>
@@ -4248,11 +4256,11 @@
         </is>
       </c>
       <c r="H153" s="6" t="n">
-        <v>-1758852</v>
+        <v>-4388718</v>
       </c>
       <c r="I153" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288453</t>
+          <t>DESCUENTO PMP1288454</t>
         </is>
       </c>
     </row>
@@ -4264,11 +4272,11 @@
       </c>
       <c r="D154" s="10" t="inlineStr">
         <is>
-          <t>PMP1288454</t>
+          <t>PMP1288455</t>
         </is>
       </c>
       <c r="E154" s="6" t="n">
-        <v>-4388718</v>
+        <v>-3480075</v>
       </c>
       <c r="F154" s="10" t="inlineStr">
         <is>
@@ -4281,11 +4289,11 @@
         </is>
       </c>
       <c r="H154" s="6" t="n">
-        <v>-4388718</v>
+        <v>-3480075</v>
       </c>
       <c r="I154" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288454</t>
+          <t>DESCUENTO PMP1288455</t>
         </is>
       </c>
     </row>
@@ -4297,11 +4305,11 @@
       </c>
       <c r="D155" s="10" t="inlineStr">
         <is>
-          <t>PMP1288455</t>
+          <t>PMP1288456</t>
         </is>
       </c>
       <c r="E155" s="6" t="n">
-        <v>-3480075</v>
+        <v>-909435</v>
       </c>
       <c r="F155" s="10" t="inlineStr">
         <is>
@@ -4314,11 +4322,11 @@
         </is>
       </c>
       <c r="H155" s="6" t="n">
-        <v>-3480075</v>
+        <v>-909435</v>
       </c>
       <c r="I155" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288455</t>
+          <t>DESCUENTO PMP1288456</t>
         </is>
       </c>
     </row>
@@ -4330,11 +4338,11 @@
       </c>
       <c r="D156" s="10" t="inlineStr">
         <is>
-          <t>PMP1288456</t>
+          <t>PMP1288803</t>
         </is>
       </c>
       <c r="E156" s="6" t="n">
-        <v>-909435</v>
+        <v>-196437</v>
       </c>
       <c r="F156" s="10" t="inlineStr">
         <is>
@@ -4347,11 +4355,11 @@
         </is>
       </c>
       <c r="H156" s="6" t="n">
-        <v>-909435</v>
+        <v>-196437</v>
       </c>
       <c r="I156" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288456</t>
+          <t>DESCUENTO PMP1288803</t>
         </is>
       </c>
     </row>
@@ -4363,11 +4371,11 @@
       </c>
       <c r="D157" s="10" t="inlineStr">
         <is>
-          <t>PMP1288803</t>
+          <t>PMP1288804</t>
         </is>
       </c>
       <c r="E157" s="6" t="n">
-        <v>-196437</v>
+        <v>-130887</v>
       </c>
       <c r="F157" s="10" t="inlineStr">
         <is>
@@ -4380,11 +4388,11 @@
         </is>
       </c>
       <c r="H157" s="6" t="n">
-        <v>-196437</v>
+        <v>-130887</v>
       </c>
       <c r="I157" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288803</t>
+          <t>DESCUENTO PMP1288804</t>
         </is>
       </c>
     </row>
@@ -4396,11 +4404,11 @@
       </c>
       <c r="D158" s="10" t="inlineStr">
         <is>
-          <t>PMP1288804</t>
+          <t>PMP1288807</t>
         </is>
       </c>
       <c r="E158" s="6" t="n">
-        <v>-130887</v>
+        <v>-229690</v>
       </c>
       <c r="F158" s="10" t="inlineStr">
         <is>
@@ -4413,11 +4421,11 @@
         </is>
       </c>
       <c r="H158" s="6" t="n">
-        <v>-130887</v>
+        <v>-229690</v>
       </c>
       <c r="I158" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288804</t>
+          <t>DESCUENTO PMP1288807</t>
         </is>
       </c>
     </row>
@@ -4429,11 +4437,11 @@
       </c>
       <c r="D159" s="10" t="inlineStr">
         <is>
-          <t>PMP1288807</t>
+          <t>PMP1288808</t>
         </is>
       </c>
       <c r="E159" s="6" t="n">
-        <v>-229690</v>
+        <v>-363261</v>
       </c>
       <c r="F159" s="10" t="inlineStr">
         <is>
@@ -4446,11 +4454,11 @@
         </is>
       </c>
       <c r="H159" s="6" t="n">
-        <v>-229690</v>
+        <v>-363261</v>
       </c>
       <c r="I159" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288807</t>
+          <t>DESCUENTO PMP1288808</t>
         </is>
       </c>
     </row>
@@ -4462,11 +4470,11 @@
       </c>
       <c r="D160" s="10" t="inlineStr">
         <is>
-          <t>PMP1288808</t>
+          <t>PMP1288809</t>
         </is>
       </c>
       <c r="E160" s="6" t="n">
-        <v>-363261</v>
+        <v>-446050</v>
       </c>
       <c r="F160" s="10" t="inlineStr">
         <is>
@@ -4479,11 +4487,11 @@
         </is>
       </c>
       <c r="H160" s="6" t="n">
-        <v>-363261</v>
+        <v>-446050</v>
       </c>
       <c r="I160" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288808</t>
+          <t>DESCUENTO PMP1288809</t>
         </is>
       </c>
     </row>
@@ -4495,11 +4503,11 @@
       </c>
       <c r="D161" s="10" t="inlineStr">
         <is>
-          <t>PMP1288809</t>
+          <t>PMP1290080</t>
         </is>
       </c>
       <c r="E161" s="6" t="n">
-        <v>-446050</v>
+        <v>-19823</v>
       </c>
       <c r="F161" s="10" t="inlineStr">
         <is>
@@ -4512,11 +4520,11 @@
         </is>
       </c>
       <c r="H161" s="6" t="n">
-        <v>-446050</v>
+        <v>-19823</v>
       </c>
       <c r="I161" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1288809</t>
+          <t>DESCUENTO PMP1290080</t>
         </is>
       </c>
     </row>
@@ -4528,11 +4536,11 @@
       </c>
       <c r="D162" s="10" t="inlineStr">
         <is>
-          <t>PMP1290080</t>
+          <t>PMP1290085</t>
         </is>
       </c>
       <c r="E162" s="6" t="n">
-        <v>-19823</v>
+        <v>-714480</v>
       </c>
       <c r="F162" s="10" t="inlineStr">
         <is>
@@ -4545,11 +4553,11 @@
         </is>
       </c>
       <c r="H162" s="6" t="n">
-        <v>-19823</v>
+        <v>-714480</v>
       </c>
       <c r="I162" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1290080</t>
+          <t>DESCUENTO PMP1290085</t>
         </is>
       </c>
     </row>
@@ -4561,11 +4569,11 @@
       </c>
       <c r="D163" s="10" t="inlineStr">
         <is>
-          <t>PMP1290085</t>
+          <t>PMP1290089</t>
         </is>
       </c>
       <c r="E163" s="6" t="n">
-        <v>-714480</v>
+        <v>-179100</v>
       </c>
       <c r="F163" s="10" t="inlineStr">
         <is>
@@ -4578,11 +4586,11 @@
         </is>
       </c>
       <c r="H163" s="6" t="n">
-        <v>-714480</v>
+        <v>-179100</v>
       </c>
       <c r="I163" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1290085</t>
+          <t>DESCUENTO PMP1290089</t>
         </is>
       </c>
     </row>
@@ -4594,11 +4602,11 @@
       </c>
       <c r="D164" s="10" t="inlineStr">
         <is>
-          <t>PMP1290089</t>
+          <t>PMP1290090</t>
         </is>
       </c>
       <c r="E164" s="6" t="n">
-        <v>-179100</v>
+        <v>-757757</v>
       </c>
       <c r="F164" s="10" t="inlineStr">
         <is>
@@ -4611,11 +4619,11 @@
         </is>
       </c>
       <c r="H164" s="6" t="n">
-        <v>-179100</v>
+        <v>-757757</v>
       </c>
       <c r="I164" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1290089</t>
+          <t>DESCUENTO PMP1290090</t>
         </is>
       </c>
     </row>
@@ -4627,11 +4635,11 @@
       </c>
       <c r="D165" s="10" t="inlineStr">
         <is>
-          <t>PMP1290090</t>
+          <t>PMP1290091</t>
         </is>
       </c>
       <c r="E165" s="6" t="n">
-        <v>-757757</v>
+        <v>-244947</v>
       </c>
       <c r="F165" s="10" t="inlineStr">
         <is>
@@ -4644,11 +4652,11 @@
         </is>
       </c>
       <c r="H165" s="6" t="n">
-        <v>-757757</v>
+        <v>-244947</v>
       </c>
       <c r="I165" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1290090</t>
+          <t>DESCUENTO PMP1290091</t>
         </is>
       </c>
     </row>
@@ -4660,11 +4668,11 @@
       </c>
       <c r="D166" s="10" t="inlineStr">
         <is>
-          <t>PMP1290091</t>
+          <t>PMP1290093</t>
         </is>
       </c>
       <c r="E166" s="6" t="n">
-        <v>-244947</v>
+        <v>-1093555</v>
       </c>
       <c r="F166" s="10" t="inlineStr">
         <is>
@@ -4677,130 +4685,130 @@
         </is>
       </c>
       <c r="H166" s="6" t="n">
-        <v>-244947</v>
+        <v>-1093555</v>
       </c>
       <c r="I166" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1290091</t>
+          <t>DESCUENTO PMP1290093</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="C167" s="10" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra</t>
+          <t>Nota</t>
         </is>
       </c>
       <c r="D167" s="10" t="inlineStr">
         <is>
-          <t>PMP1290093</t>
+          <t>C. UNILEVER</t>
         </is>
       </c>
       <c r="E167" s="6" t="n">
-        <v>-1093555</v>
+        <v>-21763968</v>
       </c>
       <c r="F167" s="10" t="inlineStr">
         <is>
-          <t>DESCUENTO</t>
+          <t>DPP NO PROCEDE</t>
         </is>
       </c>
       <c r="G167" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>667</t>
         </is>
       </c>
       <c r="H167" s="6" t="n">
-        <v>-1093555</v>
+        <v>-21763968</v>
       </c>
       <c r="I167" s="11" t="inlineStr">
         <is>
-          <t>DESCUENTO PMP1290093</t>
+          <t>DPP NO PROCEDE C. UNILEVER</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="C168" s="10" t="inlineStr">
         <is>
-          <t>Nota</t>
+          <t>Traslado Notas  Deudor acreedor</t>
         </is>
       </c>
       <c r="D168" s="10" t="inlineStr">
         <is>
-          <t>C. UNILEVER</t>
+          <t>Traslado Notas  Deudor acreedor</t>
         </is>
       </c>
       <c r="E168" s="6" t="n">
-        <v>-21763968</v>
+        <v>-522525692</v>
       </c>
       <c r="F168" s="10" t="inlineStr">
         <is>
-          <t>DPP NO PROCEDE</t>
+          <t>FACT PROVEEDOR</t>
         </is>
       </c>
       <c r="G168" s="10" t="inlineStr">
         <is>
-          <t>667</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H168" s="6" t="n">
-        <v>-21763968</v>
+        <v>-522525692</v>
       </c>
       <c r="I168" s="11" t="inlineStr">
         <is>
-          <t>DPP NO PROCEDE C. UNILEVER</t>
+          <t>FACT PROVEEDOR Traslado Notas  Deudor acreedor</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="C169" s="10" t="inlineStr">
         <is>
-          <t>Traslado Notas  Deudor acreedor</t>
+          <t>Descuento Cliente</t>
         </is>
       </c>
       <c r="D169" s="10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="E169" s="6" t="n">
-        <v>-522525692</v>
+        <v>-1181.899999991962</v>
       </c>
       <c r="F169" s="10" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="G169" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>CSR</t>
         </is>
       </c>
       <c r="H169" s="6" t="n">
-        <v>-522525692</v>
+        <v>-1181.899999991962</v>
       </c>
       <c r="I169" s="11" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR nan</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="C170" s="10" t="inlineStr">
         <is>
-          <t>Traslado proximo Pago proveedor</t>
+          <t>Nota de reintegro</t>
         </is>
       </c>
       <c r="D170" s="10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>Nota de reintegro</t>
         </is>
       </c>
       <c r="E170" s="6" t="n">
-        <v>522525692</v>
+        <v>359576835</v>
       </c>
       <c r="F170" s="10" t="inlineStr">
         <is>
-          <t>REVISAR</t>
+          <t>NOTA CLIENTE</t>
         </is>
       </c>
       <c r="G170" s="10" t="inlineStr">
@@ -4809,44 +4817,44 @@
         </is>
       </c>
       <c r="H170" s="6" t="n">
-        <v>522525692</v>
+        <v>359576835</v>
       </c>
       <c r="I170" s="11" t="inlineStr">
         <is>
-          <t>REVISAR nan</t>
+          <t>Cruza nota 1700021873 fondo inversiones 2025-Unile</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="C171" s="10" t="inlineStr">
         <is>
-          <t>Descuento Cliente</t>
+          <t>Traslado proximo Pago proveedor</t>
         </is>
       </c>
       <c r="D171" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>Traslado proximo Pago proveedor</t>
         </is>
       </c>
       <c r="E171" s="6" t="n">
-        <v>1181.899999991962</v>
+        <v>522525692</v>
       </c>
       <c r="F171" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>REVISAR</t>
         </is>
       </c>
       <c r="G171" s="10" t="inlineStr">
         <is>
-          <t>384</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H171" s="6" t="n">
-        <v>1181.899999991962</v>
+        <v>522525692</v>
       </c>
       <c r="I171" s="11" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>REVISAR Traslado proximo Pago proveedor</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cenco bien, intento de Euro
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_copi.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_copi.xlsx
@@ -584,10 +584,8 @@
           <t>Codigo de Cliente</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>10267298.0</t>
-        </is>
+      <c r="D8" s="4" t="n">
+        <v>10267298</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -630,7 +628,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>25/11/2025</t>
+          <t>01/12/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2107,7 +2105,7 @@
     <row r="71">
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>Descuento Cliente</t>
+          <t>Descuentos Clientes</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Nuevo codigo. Lectura de imagenes. Cruz Verde
</commit_message>
<xml_diff>
--- a/Pruebas/Archivos/Template/Colombia/Template_HRC_copi.xlsx
+++ b/Pruebas/Archivos/Template/Colombia/Template_HRC_copi.xlsx
@@ -628,7 +628,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>01/12/2025</t>
+          <t>05/12/2025</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -2072,82 +2072,82 @@
     <row r="70">
       <c r="C70" s="10" t="inlineStr">
         <is>
-          <t>Traslado Notas  Deudor acreedor</t>
+          <t>Nota</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
         <is>
-          <t>TR DEUDOR</t>
+          <t>Nota</t>
         </is>
       </c>
       <c r="E70" s="6" t="n">
-        <v>-7851708</v>
+        <v>-28944770</v>
       </c>
       <c r="F70" s="10" t="inlineStr">
         <is>
-          <t>Factura proveedor</t>
+          <t>Ventas</t>
         </is>
       </c>
       <c r="G70" s="10" t="inlineStr">
         <is>
-          <t>CSB</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H70" s="6" t="n">
-        <v>-7851708</v>
+        <v>-28944770</v>
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>FACT PROVEEDOR TD 36165233</t>
+          <t>SUPER SEMANAL 12-21 OCT 2025</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="C71" s="10" t="inlineStr">
         <is>
-          <t>Descuentos Clientes</t>
+          <t>Nota</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>Nota</t>
         </is>
       </c>
       <c r="E71" s="6" t="n">
-        <v>-463.6000000037311</v>
+        <v>-143553071</v>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>Ventas</t>
         </is>
       </c>
       <c r="G71" s="10" t="inlineStr">
         <is>
-          <t>CSR</t>
+          <t>987</t>
         </is>
       </c>
       <c r="H71" s="6" t="n">
-        <v>-463.6000000037311</v>
+        <v>-143553071</v>
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>MENORES VALORES</t>
+          <t>DDPD UNILEVER MIN CON 3Q 2025</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="C72" s="10" t="inlineStr">
         <is>
-          <t>Nota</t>
+          <t>Reduc Factura Compra</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
         <is>
-          <t>Nota</t>
+          <t>PMP1295578</t>
         </is>
       </c>
       <c r="E72" s="6" t="n">
-        <v>-28944770</v>
+        <v>-384234</v>
       </c>
       <c r="F72" s="10" t="inlineStr">
         <is>
@@ -2160,27 +2160,27 @@
         </is>
       </c>
       <c r="H72" s="6" t="n">
-        <v>-28944770</v>
+        <v>-384234</v>
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>SUPER SEMANAL 12-21 OCT 2025</t>
+          <t>Reduc Factura Compra PMP1295578</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="C73" s="10" t="inlineStr">
         <is>
-          <t>Nota</t>
+          <t>Reduc Factura Compra</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
         <is>
-          <t>Nota</t>
+          <t>PMP1295580</t>
         </is>
       </c>
       <c r="E73" s="6" t="n">
-        <v>-143553071</v>
+        <v>-332819</v>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
@@ -2193,11 +2193,11 @@
         </is>
       </c>
       <c r="H73" s="6" t="n">
-        <v>-143553071</v>
+        <v>-332819</v>
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>DDPD UNILEVER MIN CON 3Q 2025</t>
+          <t>Reduc Factura Compra PMP1295580</t>
         </is>
       </c>
     </row>
@@ -2209,11 +2209,11 @@
       </c>
       <c r="D74" s="10" t="inlineStr">
         <is>
-          <t>PMP1295578</t>
+          <t>PMP1295581</t>
         </is>
       </c>
       <c r="E74" s="6" t="n">
-        <v>-384234</v>
+        <v>-261572</v>
       </c>
       <c r="F74" s="10" t="inlineStr">
         <is>
@@ -2226,11 +2226,11 @@
         </is>
       </c>
       <c r="H74" s="6" t="n">
-        <v>-384234</v>
+        <v>-261572</v>
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra PMP1295578</t>
+          <t>Reduc Factura Compra PMP1295581</t>
         </is>
       </c>
     </row>
@@ -2242,11 +2242,11 @@
       </c>
       <c r="D75" s="10" t="inlineStr">
         <is>
-          <t>PMP1295580</t>
+          <t>PMP1296790</t>
         </is>
       </c>
       <c r="E75" s="6" t="n">
-        <v>-332819</v>
+        <v>-142485</v>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
@@ -2259,11 +2259,11 @@
         </is>
       </c>
       <c r="H75" s="6" t="n">
-        <v>-332819</v>
+        <v>-142485</v>
       </c>
       <c r="I75" s="11" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra PMP1295580</t>
+          <t>Reduc Factura Compra PMP1296790</t>
         </is>
       </c>
     </row>
@@ -2275,11 +2275,11 @@
       </c>
       <c r="D76" s="10" t="inlineStr">
         <is>
-          <t>PMP1295581</t>
+          <t>PMP1296791</t>
         </is>
       </c>
       <c r="E76" s="6" t="n">
-        <v>-261572</v>
+        <v>-192117</v>
       </c>
       <c r="F76" s="10" t="inlineStr">
         <is>
@@ -2292,11 +2292,11 @@
         </is>
       </c>
       <c r="H76" s="6" t="n">
-        <v>-261572</v>
+        <v>-192117</v>
       </c>
       <c r="I76" s="11" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra PMP1295581</t>
+          <t>Reduc Factura Compra PMP1296791</t>
         </is>
       </c>
     </row>
@@ -2308,11 +2308,11 @@
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>PMP1296790</t>
+          <t>PMP1296792</t>
         </is>
       </c>
       <c r="E77" s="6" t="n">
-        <v>-142485</v>
+        <v>-37602</v>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
@@ -2325,11 +2325,11 @@
         </is>
       </c>
       <c r="H77" s="6" t="n">
-        <v>-142485</v>
+        <v>-37602</v>
       </c>
       <c r="I77" s="11" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra PMP1296790</t>
+          <t>Reduc Factura Compra PMP1296792</t>
         </is>
       </c>
     </row>
@@ -2341,11 +2341,11 @@
       </c>
       <c r="D78" s="10" t="inlineStr">
         <is>
-          <t>PMP1296791</t>
+          <t>PMP1299325</t>
         </is>
       </c>
       <c r="E78" s="6" t="n">
-        <v>-192117</v>
+        <v>-864841</v>
       </c>
       <c r="F78" s="10" t="inlineStr">
         <is>
@@ -2358,11 +2358,11 @@
         </is>
       </c>
       <c r="H78" s="6" t="n">
-        <v>-192117</v>
+        <v>-864841</v>
       </c>
       <c r="I78" s="11" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra PMP1296791</t>
+          <t>Reduc Factura Compra PMP1299325</t>
         </is>
       </c>
     </row>
@@ -2374,11 +2374,11 @@
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>PMP1296792</t>
+          <t>PMP1299326</t>
         </is>
       </c>
       <c r="E79" s="6" t="n">
-        <v>-37602</v>
+        <v>-967635</v>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
@@ -2391,11 +2391,11 @@
         </is>
       </c>
       <c r="H79" s="6" t="n">
-        <v>-37602</v>
+        <v>-967635</v>
       </c>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra PMP1296792</t>
+          <t>Reduc Factura Compra PMP1299326</t>
         </is>
       </c>
     </row>
@@ -2407,11 +2407,11 @@
       </c>
       <c r="D80" s="10" t="inlineStr">
         <is>
-          <t>PMP1299325</t>
+          <t>PMP1299331</t>
         </is>
       </c>
       <c r="E80" s="6" t="n">
-        <v>-864841</v>
+        <v>-1056</v>
       </c>
       <c r="F80" s="10" t="inlineStr">
         <is>
@@ -2424,77 +2424,77 @@
         </is>
       </c>
       <c r="H80" s="6" t="n">
-        <v>-864841</v>
+        <v>-1056</v>
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra PMP1299325</t>
+          <t>Reduc Factura Compra PMP1299331</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="C81" s="10" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra</t>
+          <t>Traslado Notas  Deudor acreedor</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>PMP1299326</t>
+          <t>TR DEUDOR</t>
         </is>
       </c>
       <c r="E81" s="6" t="n">
-        <v>-967635</v>
+        <v>-7851708</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
-          <t>Ventas</t>
+          <t>Factura proveedor</t>
         </is>
       </c>
       <c r="G81" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>CSB</t>
         </is>
       </c>
       <c r="H81" s="6" t="n">
-        <v>-967635</v>
+        <v>-7851708</v>
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra PMP1299326</t>
+          <t>FACT PROVEEDOR TD 36165233</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="C82" s="10" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra</t>
+          <t>Descuentos Clientes</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>PMP1299331</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="E82" s="6" t="n">
-        <v>-1056</v>
+        <v>-463.6000000037311</v>
       </c>
       <c r="F82" s="10" t="inlineStr">
         <is>
-          <t>Ventas</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
       <c r="G82" s="10" t="inlineStr">
         <is>
-          <t>987</t>
+          <t>CSR</t>
         </is>
       </c>
       <c r="H82" s="6" t="n">
-        <v>-1056</v>
+        <v>-463.6000000037311</v>
       </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>Reduc Factura Compra PMP1299331</t>
+          <t>MENORES VALORES</t>
         </is>
       </c>
     </row>

</xml_diff>